<commit_message>
Celcat kontrolü: nochange (2026-10-26)
</commit_message>
<xml_diff>
--- a/docs/lodz-ders-programi.xlsx
+++ b/docs/lodz-ders-programi.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Değişiklikler" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Haftalık Şablon" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tüm Dersler" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grup Seçimleri" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notlar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Değişiklikler" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Haftalık Şablon" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tüm Dersler" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Grup Seçimleri" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notlar" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Haftalık Şablon'!$A$1:$J$23</definedName>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -573,100 +573,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>26.10.2026 14:54</t>
+          <t>26.10.2026 14:59</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Celcat'ta senin derslerinde 11 değişiklik var:</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>DEĞİŞTİ: Production Management Methods Laboratory (3BSTen/fr - ERASMUS 1) | Pzt 10:15–12:00, 11 tarih: 26 Eki, 2 Kas, 16 Kas, 23 Kas, 30 Kas, 7 Ara, 14 Ara, 21 Ara, 11 Oca, 18 Oca, 25 Oca | IFE (A-16) · 103  [salon IFE (A-16) · 12 → IFE (A-16) · 103]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Production Management Methods Laboratory (3BSTen/fr - ERASMUS 1) – FACTORY VISIT 1 – BSH | 3 Kas Sal 11:00–13:00 | Yer: hocadan öğren (salon yok)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Production Management Methods Laboratory (3BSTen/fr - ERASMUS 1) – The White Factory - trip | 20 Kas Cum 10:00–12:15 | Yer: hocadan öğren (salon yok)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>DEĞİŞTİ: Production Management Methods Lecture | 4 Ara Cum 14:15–18:15 | A22 · 1M02  [önceden 14:15–15:45, A22 · 1M02]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Production Management Methods Laboratory (3BSTen/fr - ERASMUS 1) | 1 Şub Pzt 10:15–12:00 | IFE (A-16) · 103</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Machine Learning Lecture | 1 Şub Pzt 14:15–15:45 | B14 · 2.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Machine Learning Project (5MMDA - group 1) | 1 Şub Pzt 16:15–17:45 | B14 · 2.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Cloud Computing Systems Project (5IT - ERASMUS 1, 5IT - ERASMUS 2) | 1 Şub Pzt 18:00–19:30 | B19 · 103</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Cloud Computing Systems Lecture | 2 Şub Sal 10:15–11:45 | B9 · F2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Digital Systems 1 Laboratory (3CS - ERASMUS) | 2 Şub Sal 12:15–13:45 | B9/i23 · 204</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>YENİ: Information Technologies Laboratory (1ETE - group 2) | 2 Şub Sal 17:15–19:45 | B18 · lab.B</t>
+          <t>Senin derslerinde değişiklik yok.</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11338,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>26.10.2026 14:54</t>
+          <t>26.10.2026 14:59</t>
         </is>
       </c>
     </row>

</xml_diff>